<commit_message>
Daily generated and validated data
</commit_message>
<xml_diff>
--- a/decision_log.xlsx
+++ b/decision_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K551"/>
+  <dimension ref="A1:K601"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26032,7 +26032,7 @@
         </is>
       </c>
       <c r="J502" s="2" t="n">
-        <v>46087.53937713445</v>
+        <v>46087.53937712963</v>
       </c>
       <c r="K502" t="inlineStr">
         <is>
@@ -26083,7 +26083,7 @@
         </is>
       </c>
       <c r="J503" s="2" t="n">
-        <v>46088.4560438054</v>
+        <v>46088.45604380787</v>
       </c>
       <c r="K503" t="inlineStr">
         <is>
@@ -26134,7 +26134,7 @@
         </is>
       </c>
       <c r="J504" s="2" t="n">
-        <v>46064.33104380868</v>
+        <v>46064.33104380787</v>
       </c>
       <c r="K504" t="inlineStr">
         <is>
@@ -26185,7 +26185,7 @@
         </is>
       </c>
       <c r="J505" s="2" t="n">
-        <v>46065.49771047864</v>
+        <v>46065.49771047453</v>
       </c>
       <c r="K505" t="inlineStr">
         <is>
@@ -26236,7 +26236,7 @@
         </is>
       </c>
       <c r="J506" s="2" t="n">
-        <v>46070.66437714858</v>
+        <v>46070.66437715277</v>
       </c>
       <c r="K506" t="inlineStr">
         <is>
@@ -26287,7 +26287,7 @@
         </is>
       </c>
       <c r="J507" s="2" t="n">
-        <v>46059.53937715171</v>
+        <v>46059.53937715277</v>
       </c>
       <c r="K507" t="inlineStr">
         <is>
@@ -26338,7 +26338,7 @@
         </is>
       </c>
       <c r="J508" s="2" t="n">
-        <v>46070.53937715492</v>
+        <v>46070.53937715277</v>
       </c>
       <c r="K508" t="inlineStr">
         <is>
@@ -26389,7 +26389,7 @@
         </is>
       </c>
       <c r="J509" s="2" t="n">
-        <v>46061.33104382484</v>
+        <v>46061.33104381945</v>
       </c>
       <c r="K509" t="inlineStr">
         <is>
@@ -26440,7 +26440,7 @@
         </is>
       </c>
       <c r="J510" s="2" t="n">
-        <v>46088.41437716169</v>
+        <v>46088.41437716435</v>
       </c>
       <c r="K510" t="inlineStr">
         <is>
@@ -26491,7 +26491,7 @@
         </is>
       </c>
       <c r="J511" s="2" t="n">
-        <v>46081.49771049835</v>
+        <v>46081.49771049769</v>
       </c>
       <c r="K511" t="inlineStr">
         <is>
@@ -26542,7 +26542,7 @@
         </is>
       </c>
       <c r="J512" s="2" t="n">
-        <v>46065.4143771681</v>
+        <v>46065.41437716435</v>
       </c>
       <c r="K512" t="inlineStr">
         <is>
@@ -26593,7 +26593,7 @@
         </is>
       </c>
       <c r="J513" s="2" t="n">
-        <v>46085.70604383809</v>
+        <v>46085.70604384259</v>
       </c>
       <c r="K513" t="inlineStr">
         <is>
@@ -26644,7 +26644,7 @@
         </is>
       </c>
       <c r="J514" s="2" t="n">
-        <v>46067.37271050802</v>
+        <v>46067.37271050926</v>
       </c>
       <c r="K514" t="inlineStr">
         <is>
@@ -26695,7 +26695,7 @@
         </is>
       </c>
       <c r="J515" s="2" t="n">
-        <v>46088.58104384453</v>
+        <v>46088.58104384259</v>
       </c>
       <c r="K515" t="inlineStr">
         <is>
@@ -26746,7 +26746,7 @@
         </is>
       </c>
       <c r="J516" s="2" t="n">
-        <v>46076.62271051436</v>
+        <v>46076.62271050926</v>
       </c>
       <c r="K516" t="inlineStr">
         <is>
@@ -26797,7 +26797,7 @@
         </is>
       </c>
       <c r="J517" s="2" t="n">
-        <v>46075.37271051761</v>
+        <v>46075.37271052083</v>
       </c>
       <c r="K517" t="inlineStr">
         <is>
@@ -26848,7 +26848,7 @@
         </is>
       </c>
       <c r="J518" s="2" t="n">
-        <v>46066.41437718735</v>
+        <v>46066.4143771875</v>
       </c>
       <c r="K518" t="inlineStr">
         <is>
@@ -26899,7 +26899,7 @@
         </is>
       </c>
       <c r="J519" s="2" t="n">
-        <v>46067.53937719043</v>
+        <v>46067.5393771875</v>
       </c>
       <c r="K519" t="inlineStr">
         <is>
@@ -26950,7 +26950,7 @@
         </is>
       </c>
       <c r="J520" s="2" t="n">
-        <v>46059.33104386034</v>
+        <v>46059.33104386574</v>
       </c>
       <c r="K520" t="inlineStr">
         <is>
@@ -27001,7 +27001,7 @@
         </is>
       </c>
       <c r="J521" s="2" t="n">
-        <v>46064.4560438634</v>
+        <v>46064.45604386574</v>
       </c>
       <c r="K521" t="inlineStr">
         <is>
@@ -27052,7 +27052,7 @@
         </is>
       </c>
       <c r="J522" s="2" t="n">
-        <v>46082.62271053311</v>
+        <v>46082.62271053241</v>
       </c>
       <c r="K522" t="inlineStr">
         <is>
@@ -27103,7 +27103,7 @@
         </is>
       </c>
       <c r="J523" s="2" t="n">
-        <v>46076.45604386947</v>
+        <v>46076.45604386574</v>
       </c>
       <c r="K523" t="inlineStr">
         <is>
@@ -27154,7 +27154,7 @@
         </is>
       </c>
       <c r="J524" s="2" t="n">
-        <v>46071.53937720609</v>
+        <v>46071.53937721065</v>
       </c>
       <c r="K524" t="inlineStr">
         <is>
@@ -27205,7 +27205,7 @@
         </is>
       </c>
       <c r="J525" s="2" t="n">
-        <v>46077.66437720925</v>
+        <v>46077.66437721065</v>
       </c>
       <c r="K525" t="inlineStr">
         <is>
@@ -27256,7 +27256,7 @@
         </is>
       </c>
       <c r="J526" s="2" t="n">
-        <v>46088.66437721228</v>
+        <v>46088.66437721065</v>
       </c>
       <c r="K526" t="inlineStr">
         <is>
@@ -27307,7 +27307,7 @@
         </is>
       </c>
       <c r="J527" s="2" t="n">
-        <v>46085.53937721553</v>
+        <v>46085.53937721065</v>
       </c>
       <c r="K527" t="inlineStr">
         <is>
@@ -27358,7 +27358,7 @@
         </is>
       </c>
       <c r="J528" s="2" t="n">
-        <v>46079.41437721903</v>
+        <v>46079.41437722222</v>
       </c>
       <c r="K528" t="inlineStr">
         <is>
@@ -27409,7 +27409,7 @@
         </is>
       </c>
       <c r="J529" s="2" t="n">
-        <v>46084.49771055547</v>
+        <v>46084.49771055556</v>
       </c>
       <c r="K529" t="inlineStr">
         <is>
@@ -27460,7 +27460,7 @@
         </is>
       </c>
       <c r="J530" s="2" t="n">
-        <v>46061.37271055861</v>
+        <v>46061.37271055556</v>
       </c>
       <c r="K530" t="inlineStr">
         <is>
@@ -27511,7 +27511,7 @@
         </is>
       </c>
       <c r="J531" s="2" t="n">
-        <v>46078.66437722873</v>
+        <v>46078.6643772338</v>
       </c>
       <c r="K531" t="inlineStr">
         <is>
@@ -27562,7 +27562,7 @@
         </is>
       </c>
       <c r="J532" s="2" t="n">
-        <v>46061.62271056515</v>
+        <v>46061.62271056713</v>
       </c>
       <c r="K532" t="inlineStr">
         <is>
@@ -27613,7 +27613,7 @@
         </is>
       </c>
       <c r="J533" s="2" t="n">
-        <v>46069.3727105682</v>
+        <v>46069.37271056713</v>
       </c>
       <c r="K533" t="inlineStr">
         <is>
@@ -27664,7 +27664,7 @@
         </is>
       </c>
       <c r="J534" s="2" t="n">
-        <v>46076.33104390463</v>
+        <v>46076.33104390046</v>
       </c>
       <c r="K534" t="inlineStr">
         <is>
@@ -27715,7 +27715,7 @@
         </is>
       </c>
       <c r="J535" s="2" t="n">
-        <v>46071.49771057453</v>
+        <v>46071.4977105787</v>
       </c>
       <c r="K535" t="inlineStr">
         <is>
@@ -27766,7 +27766,7 @@
         </is>
       </c>
       <c r="J536" s="2" t="n">
-        <v>46082.70604391103</v>
+        <v>46082.70604391204</v>
       </c>
       <c r="K536" t="inlineStr">
         <is>
@@ -27817,7 +27817,7 @@
         </is>
       </c>
       <c r="J537" s="2" t="n">
-        <v>46062.33104391408</v>
+        <v>46062.33104391204</v>
       </c>
       <c r="K537" t="inlineStr">
         <is>
@@ -27868,7 +27868,7 @@
         </is>
       </c>
       <c r="J538" s="2" t="n">
-        <v>46068.41437725046</v>
+        <v>46068.41437724537</v>
       </c>
       <c r="K538" t="inlineStr">
         <is>
@@ -27919,7 +27919,7 @@
         </is>
       </c>
       <c r="J539" s="2" t="n">
-        <v>46061.33104392058</v>
+        <v>46061.33104392361</v>
       </c>
       <c r="K539" t="inlineStr">
         <is>
@@ -27970,7 +27970,7 @@
         </is>
       </c>
       <c r="J540" s="2" t="n">
-        <v>46064.33104392376</v>
+        <v>46064.33104392361</v>
       </c>
       <c r="K540" t="inlineStr">
         <is>
@@ -28021,7 +28021,7 @@
         </is>
       </c>
       <c r="J541" s="2" t="n">
-        <v>46073.7060439268</v>
+        <v>46073.70604392361</v>
       </c>
       <c r="K541" t="inlineStr">
         <is>
@@ -28072,7 +28072,7 @@
         </is>
       </c>
       <c r="J542" s="2" t="n">
-        <v>46072.53937726333</v>
+        <v>46072.53937726852</v>
       </c>
       <c r="K542" t="inlineStr">
         <is>
@@ -28123,7 +28123,7 @@
         </is>
       </c>
       <c r="J543" s="2" t="n">
-        <v>46078.70604393321</v>
+        <v>46078.70604393518</v>
       </c>
       <c r="K543" t="inlineStr">
         <is>
@@ -28174,7 +28174,7 @@
         </is>
       </c>
       <c r="J544" s="2" t="n">
-        <v>46070.4143772696</v>
+        <v>46070.41437726852</v>
       </c>
       <c r="K544" t="inlineStr">
         <is>
@@ -28225,7 +28225,7 @@
         </is>
       </c>
       <c r="J545" s="2" t="n">
-        <v>46070.3310439393</v>
+        <v>46070.33104393518</v>
       </c>
       <c r="K545" t="inlineStr">
         <is>
@@ -28276,7 +28276,7 @@
         </is>
       </c>
       <c r="J546" s="2" t="n">
-        <v>46060.66437727593</v>
+        <v>46060.66437728009</v>
       </c>
       <c r="K546" t="inlineStr">
         <is>
@@ -28327,7 +28327,7 @@
         </is>
       </c>
       <c r="J547" s="2" t="n">
-        <v>46071.4977106123</v>
+        <v>46071.49771061342</v>
       </c>
       <c r="K547" t="inlineStr">
         <is>
@@ -28378,7 +28378,7 @@
         </is>
       </c>
       <c r="J548" s="2" t="n">
-        <v>46080.45604394881</v>
+        <v>46080.45604394676</v>
       </c>
       <c r="K548" t="inlineStr">
         <is>
@@ -28429,7 +28429,7 @@
         </is>
       </c>
       <c r="J549" s="2" t="n">
-        <v>46084.45604395191</v>
+        <v>46084.45604394676</v>
       </c>
       <c r="K549" t="inlineStr">
         <is>
@@ -28480,7 +28480,7 @@
         </is>
       </c>
       <c r="J550" s="2" t="n">
-        <v>46066.62271062179</v>
+        <v>46066.622710625</v>
       </c>
       <c r="K550" t="inlineStr">
         <is>
@@ -28531,11 +28531,2561 @@
         </is>
       </c>
       <c r="J551" s="2" t="n">
-        <v>46061.33104395819</v>
+        <v>46061.33104395834</v>
       </c>
       <c r="K551" t="inlineStr">
         <is>
           <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>24815e3c-61d8-42d3-8f88-c131984358a2</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>857d0806-0f10-4330-b2ed-de37b27b20a9</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D552" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E552" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="F552" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G552" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H552" t="inlineStr">
+        <is>
+          <t>OP-352</t>
+        </is>
+      </c>
+      <c r="I552" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J552" s="2" t="n">
+        <v>46060.7129640142</v>
+      </c>
+      <c r="K552" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>fae86374-d5b0-420a-a523-28571025cd18</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>eb4f135f-8fa3-4324-93b0-bf69a241c5ac</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D553" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E553" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F553" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G553" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H553" t="inlineStr">
+        <is>
+          <t>OP-981</t>
+        </is>
+      </c>
+      <c r="I553" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J553" s="2" t="n">
+        <v>46081.87963068551</v>
+      </c>
+      <c r="K553" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>83b0d62c-93d7-4cc4-abf7-1d641576bdd1</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>6c633a38-fa58-48b4-84a9-cde12968c4af</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D554" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E554" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F554" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G554" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H554" t="inlineStr">
+        <is>
+          <t>OP-120</t>
+        </is>
+      </c>
+      <c r="I554" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J554" s="2" t="n">
+        <v>46067.79629735544</v>
+      </c>
+      <c r="K554" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>e489e479-5a0c-497b-9d90-affe88219713</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>d7f36b98-11ed-4cbb-bb59-667f7df12f6a</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D555" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E555" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F555" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G555" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H555" t="inlineStr">
+        <is>
+          <t>OP-932</t>
+        </is>
+      </c>
+      <c r="I555" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J555" s="2" t="n">
+        <v>46069.62963069205</v>
+      </c>
+      <c r="K555" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>52a587ad-7ec3-43f5-a0a6-d0b609abf526</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>b74b4d9e-99cc-49de-9026-9be19d543019</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D556" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E556" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="F556" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G556" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H556" t="inlineStr">
+        <is>
+          <t>OP-710</t>
+        </is>
+      </c>
+      <c r="I556" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J556" s="2" t="n">
+        <v>46079.96296402877</v>
+      </c>
+      <c r="K556" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>3e40673d-d1ac-4930-b7bf-50f41467bb5b</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>9445f8fd-7161-4c7f-8fea-4db374579ad8</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D557" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E557" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="F557" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G557" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H557" t="inlineStr">
+        <is>
+          <t>OP-988</t>
+        </is>
+      </c>
+      <c r="I557" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J557" s="2" t="n">
+        <v>46064.7962973658</v>
+      </c>
+      <c r="K557" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>7e298f86-f90b-43be-bc93-137a9415c00c</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>f6fed973-70e2-4efe-a175-86f338d5d1b4</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D558" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E558" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="F558" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G558" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H558" t="inlineStr">
+        <is>
+          <t>OP-444</t>
+        </is>
+      </c>
+      <c r="I558" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J558" s="2" t="n">
+        <v>46076.75463070224</v>
+      </c>
+      <c r="K558" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>42038056-12d0-4d66-aad3-ef6daa90a89c</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>51628fa4-128b-42ab-9dfa-66d55d3213f1</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D559" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E559" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F559" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G559" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H559" t="inlineStr">
+        <is>
+          <t>OP-115</t>
+        </is>
+      </c>
+      <c r="I559" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J559" s="2" t="n">
+        <v>46077.67129737206</v>
+      </c>
+      <c r="K559" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>05c868e8-03c2-422f-81fa-e8d2662229c1</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>b1c8d170-cc99-40af-a96d-6635ca9be7d2</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D560" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E560" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F560" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G560" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H560" t="inlineStr">
+        <is>
+          <t>OP-860</t>
+        </is>
+      </c>
+      <c r="I560" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J560" s="2" t="n">
+        <v>46088.67129737534</v>
+      </c>
+      <c r="K560" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>93803369-433b-4414-958a-35bf790e9ffa</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>61360ffd-a88c-4ad0-a464-3a300c2c0aab</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D561" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E561" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="F561" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G561" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H561" t="inlineStr">
+        <is>
+          <t>OP-567</t>
+        </is>
+      </c>
+      <c r="I561" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J561" s="2" t="n">
+        <v>46069.79629737847</v>
+      </c>
+      <c r="K561" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>f7ccb211-b2ea-4957-a530-3a0bbeb9c352</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>09a58def-7756-4ede-9f0a-af3b60374bd7</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D562" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E562" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F562" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G562" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H562" t="inlineStr">
+        <is>
+          <t>OP-354</t>
+        </is>
+      </c>
+      <c r="I562" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J562" s="2" t="n">
+        <v>46077.87963071529</v>
+      </c>
+      <c r="K562" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>c716eabc-5253-4abd-9eb4-089d0aa24d37</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>c0bb005f-031d-45b9-ae7b-7849d437915c</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D563" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E563" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="F563" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G563" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H563" t="inlineStr">
+        <is>
+          <t>OP-532</t>
+        </is>
+      </c>
+      <c r="I563" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J563" s="2" t="n">
+        <v>46059.62963071837</v>
+      </c>
+      <c r="K563" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>c8bd0d0c-d716-4767-ab9b-46168ae1528c</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>71bad39d-82c4-4838-8ba5-50e0e33b7f01</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D564" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E564" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F564" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G564" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H564" t="inlineStr">
+        <is>
+          <t>OP-553</t>
+        </is>
+      </c>
+      <c r="I564" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J564" s="2" t="n">
+        <v>46071.79629738865</v>
+      </c>
+      <c r="K564" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>d31bbcb7-5737-4bcf-b299-789d6ea1ab3c</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>b875e5c8-7728-412d-9b81-f2e669aa7ff0</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D565" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E565" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F565" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G565" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H565" t="inlineStr">
+        <is>
+          <t>OP-846</t>
+        </is>
+      </c>
+      <c r="I565" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J565" s="2" t="n">
+        <v>46079.7129640584</v>
+      </c>
+      <c r="K565" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>e97182b7-d6ec-4606-91d6-8bdcadaf3f3d</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>fa40a6ee-08f8-417d-a633-a760fad3092b</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D566" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E566" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="F566" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G566" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H566" t="inlineStr">
+        <is>
+          <t>OP-293</t>
+        </is>
+      </c>
+      <c r="I566" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J566" s="2" t="n">
+        <v>46087.6712973949</v>
+      </c>
+      <c r="K566" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>e0410413-8bd9-4edc-bc81-d5d50ac7fb72</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>e4333b0f-b2a4-4be8-9efb-44e28f82761e</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E567" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F567" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G567" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H567" t="inlineStr">
+        <is>
+          <t>OP-579</t>
+        </is>
+      </c>
+      <c r="I567" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J567" s="2" t="n">
+        <v>46067.96296406501</v>
+      </c>
+      <c r="K567" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>013a9320-8eeb-40fc-93b8-5f68b1166b49</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>f88ba1b0-f075-43ff-8aa2-4f366bf9b2eb</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E568" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="F568" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G568" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H568" t="inlineStr">
+        <is>
+          <t>OP-918</t>
+        </is>
+      </c>
+      <c r="I568" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J568" s="2" t="n">
+        <v>46084.75463073562</v>
+      </c>
+      <c r="K568" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>f6b5275c-803b-43d7-9bc4-53d72107c388</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>fd95471f-48b8-4311-a108-ed46dca8e2b2</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E569" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="F569" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G569" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H569" t="inlineStr">
+        <is>
+          <t>OP-332</t>
+        </is>
+      </c>
+      <c r="I569" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J569" s="2" t="n">
+        <v>46073.6712974054</v>
+      </c>
+      <c r="K569" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>bd16bc06-8c11-4273-9bc5-b67fa76b4aaa</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>11e37fbf-706a-4ad0-b9bd-134a2bbdcf03</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E570" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="F570" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G570" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H570" t="inlineStr">
+        <is>
+          <t>OP-209</t>
+        </is>
+      </c>
+      <c r="I570" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J570" s="2" t="n">
+        <v>46075.9629640752</v>
+      </c>
+      <c r="K570" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>ccaa21a1-918e-451f-b45b-d5a1953a2b60</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>050659a0-ca13-4690-bd39-f6d0fe86ccbc</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E571" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F571" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G571" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H571" t="inlineStr">
+        <is>
+          <t>OP-363</t>
+        </is>
+      </c>
+      <c r="I571" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J571" s="2" t="n">
+        <v>46059.79629741182</v>
+      </c>
+      <c r="K571" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>b2f766d3-54ea-4dea-8788-a1987cf3ea90</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>3decbe6f-feb8-4242-9aac-1efb05f7a6ed</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E572" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F572" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G572" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H572" t="inlineStr">
+        <is>
+          <t>OP-126</t>
+        </is>
+      </c>
+      <c r="I572" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J572" s="2" t="n">
+        <v>46071.75463074828</v>
+      </c>
+      <c r="K572" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>7381c3ce-c847-40e6-81d7-60b96e1f0610</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>75620955-b8a1-4cfd-b93d-3737aa4e4ca1</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E573" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="F573" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G573" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>OP-230</t>
+        </is>
+      </c>
+      <c r="I573" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J573" s="2" t="n">
+        <v>46084.58796408487</v>
+      </c>
+      <c r="K573" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>dbe1fee2-e72d-4dba-aa36-544c6d6fc249</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>cf99d64b-36dd-4621-9f62-d18c7be066c1</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E574" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F574" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="G574" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H574" t="inlineStr">
+        <is>
+          <t>OP-382</t>
+        </is>
+      </c>
+      <c r="I574" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J574" s="2" t="n">
+        <v>46083.87963075478</v>
+      </c>
+      <c r="K574" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>7670eb57-217c-400d-ae35-21e7255f4647</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>43351dfe-fa9b-4f09-be50-a716542d3a47</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E575" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F575" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G575" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H575" t="inlineStr">
+        <is>
+          <t>OP-632</t>
+        </is>
+      </c>
+      <c r="I575" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J575" s="2" t="n">
+        <v>46067.71296409134</v>
+      </c>
+      <c r="K575" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>322fac2c-352f-402e-9a42-d176e4ce1370</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>0be1c8d4-3702-47dd-a82d-9014c688e352</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E576" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F576" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G576" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H576" t="inlineStr">
+        <is>
+          <t>OP-928</t>
+        </is>
+      </c>
+      <c r="I576" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J576" s="2" t="n">
+        <v>46069.96296409442</v>
+      </c>
+      <c r="K576" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>ac3e77d5-307c-4a66-8389-3c9c104179af</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>352bc9c0-e473-4f44-9c4e-34e92f74c107</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E577" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="F577" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G577" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H577" t="inlineStr">
+        <is>
+          <t>OP-538</t>
+        </is>
+      </c>
+      <c r="I577" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J577" s="2" t="n">
+        <v>46079.58796409767</v>
+      </c>
+      <c r="K577" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>695c982e-0a1e-467d-b679-6a87a4e8fe4a</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>c1353d4a-e856-4a88-98f9-f735cab6e869</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D578" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E578" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F578" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G578" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H578" t="inlineStr">
+        <is>
+          <t>OP-510</t>
+        </is>
+      </c>
+      <c r="I578" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J578" s="2" t="n">
+        <v>46071.83796410132</v>
+      </c>
+      <c r="K578" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>0f5bf304-edff-4527-8c9a-393c36a471aa</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>87626a0e-0c5e-4d23-8538-1eb671eaa3a7</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D579" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E579" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="F579" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G579" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H579" t="inlineStr">
+        <is>
+          <t>OP-205</t>
+        </is>
+      </c>
+      <c r="I579" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J579" s="2" t="n">
+        <v>46067.83796410452</v>
+      </c>
+      <c r="K579" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>b3160cbb-48cc-4d17-9107-0aac477cef39</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>5e2d5d1c-9749-4099-829b-fcf41f7754cb</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D580" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E580" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F580" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="G580" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H580" t="inlineStr">
+        <is>
+          <t>OP-922</t>
+        </is>
+      </c>
+      <c r="I580" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J580" s="2" t="n">
+        <v>46086.71296410758</v>
+      </c>
+      <c r="K580" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>2bb584b6-3b9d-4fa5-94cc-2b05155f636b</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>7a3042fb-ac42-468c-ae74-471addfd3050</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D581" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E581" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="F581" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G581" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H581" t="inlineStr">
+        <is>
+          <t>OP-347</t>
+        </is>
+      </c>
+      <c r="I581" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J581" s="2" t="n">
+        <v>46066.83796411066</v>
+      </c>
+      <c r="K581" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>b2aeec7a-08c1-498f-a2be-d76e12b5031d</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>a2b947cd-5653-42d6-933d-dd5fdecb4f6c</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D582" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E582" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="F582" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G582" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H582" t="inlineStr">
+        <is>
+          <t>OP-766</t>
+        </is>
+      </c>
+      <c r="I582" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J582" s="2" t="n">
+        <v>46088.62963078083</v>
+      </c>
+      <c r="K582" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>2ebfd676-5ffb-42b9-af30-c15a0ff89ae3</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>642f472d-2963-4870-a708-3e6cfe013157</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D583" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E583" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F583" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G583" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H583" t="inlineStr">
+        <is>
+          <t>OP-608</t>
+        </is>
+      </c>
+      <c r="I583" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J583" s="2" t="n">
+        <v>46076.67129745054</v>
+      </c>
+      <c r="K583" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>f31a5a64-b3df-4a30-93eb-1fc2624b5c37</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>d78c8701-5c91-491d-960e-fa7e50fc5f95</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D584" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E584" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="F584" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="G584" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H584" t="inlineStr">
+        <is>
+          <t>OP-445</t>
+        </is>
+      </c>
+      <c r="I584" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J584" s="2" t="n">
+        <v>46067.62963078706</v>
+      </c>
+      <c r="K584" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>a1c8f1fc-9db5-4077-91a4-35b2559b357d</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>3c4bda8b-4d61-470f-81bc-ac3410ffb05a</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E585" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="F585" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G585" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H585" t="inlineStr">
+        <is>
+          <t>OP-400</t>
+        </is>
+      </c>
+      <c r="I585" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J585" s="2" t="n">
+        <v>46073.83796412372</v>
+      </c>
+      <c r="K585" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>6209319f-c786-46b5-89ca-ba83040af8c4</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>b39f60fd-2d5e-4745-a505-349e3c08912b</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D586" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E586" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F586" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G586" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H586" t="inlineStr">
+        <is>
+          <t>OP-162</t>
+        </is>
+      </c>
+      <c r="I586" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J586" s="2" t="n">
+        <v>46075.8796307936</v>
+      </c>
+      <c r="K586" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>24e13c69-03f4-47ef-bf01-e07345571403</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>3bad2eb8-0e7a-4958-a82e-45ee1cfa3e75</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E587" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="F587" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G587" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H587" t="inlineStr">
+        <is>
+          <t>OP-839</t>
+        </is>
+      </c>
+      <c r="I587" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J587" s="2" t="n">
+        <v>46062.83796413003</v>
+      </c>
+      <c r="K587" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>bd2b9f33-9c3d-4a8d-9026-d48319b5bdce</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>4c0c5e7f-1307-49b9-a3fc-37bafcd1ec64</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D588" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E588" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F588" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G588" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H588" t="inlineStr">
+        <is>
+          <t>OP-717</t>
+        </is>
+      </c>
+      <c r="I588" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J588" s="2" t="n">
+        <v>46069.9212974664</v>
+      </c>
+      <c r="K588" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>2f01fcbe-1430-40dc-b76c-db5103d11a56</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>fc1bb941-e2a7-434a-86fb-c9d476559f3f</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E589" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F589" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G589" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H589" t="inlineStr">
+        <is>
+          <t>OP-107</t>
+        </is>
+      </c>
+      <c r="I589" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J589" s="2" t="n">
+        <v>46074.58796413642</v>
+      </c>
+      <c r="K589" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>5fa92fab-217e-437d-ac30-830e4a10823d</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>2743224a-c38b-45fe-b4af-bd238ef77cdb</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E590" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F590" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G590" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>OP-964</t>
+        </is>
+      </c>
+      <c r="I590" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J590" s="2" t="n">
+        <v>46088.96296413954</v>
+      </c>
+      <c r="K590" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>8f8e5955-11aa-4528-9bb7-b93018f5f2f2</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>0d34b840-4a4b-42cc-8f1a-25de96dc0458</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E591" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="F591" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G591" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H591" t="inlineStr">
+        <is>
+          <t>OP-397</t>
+        </is>
+      </c>
+      <c r="I591" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J591" s="2" t="n">
+        <v>46075.96296414261</v>
+      </c>
+      <c r="K591" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>3724593d-a100-4627-999f-808ccb621b3c</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>953f8dd7-1efc-4020-bbc7-4f1fab2a68ee</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E592" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F592" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G592" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H592" t="inlineStr">
+        <is>
+          <t>OP-176</t>
+        </is>
+      </c>
+      <c r="I592" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J592" s="2" t="n">
+        <v>46083.62963081271</v>
+      </c>
+      <c r="K592" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>f77c014f-9fbb-48ae-89ef-494f3ff02134</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>55744d16-dd40-4b24-a479-2241a1e83a67</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E593" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="F593" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="G593" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H593" t="inlineStr">
+        <is>
+          <t>OP-910</t>
+        </is>
+      </c>
+      <c r="I593" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J593" s="2" t="n">
+        <v>46062.79629748264</v>
+      </c>
+      <c r="K593" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>2b6e1817-ea08-47a3-9a68-0877271acf1d</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>77beae8d-b1ff-449c-9e6c-ee5fe115b020</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E594" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F594" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G594" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H594" t="inlineStr">
+        <is>
+          <t>OP-284</t>
+        </is>
+      </c>
+      <c r="I594" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J594" s="2" t="n">
+        <v>46073.79629748569</v>
+      </c>
+      <c r="K594" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>c0023e09-2b6c-4f35-9027-73e30f4d7a66</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>cc659dc5-0296-485a-979d-074e4b27294d</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E595" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="F595" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G595" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H595" t="inlineStr">
+        <is>
+          <t>OP-494</t>
+        </is>
+      </c>
+      <c r="I595" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J595" s="2" t="n">
+        <v>46075.75463082219</v>
+      </c>
+      <c r="K595" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>27cd7466-9774-4f57-abd4-2137cb1b18af</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>669b8b1a-0341-428d-97a3-b4e7169f7cd0</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E596" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="F596" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G596" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H596" t="inlineStr">
+        <is>
+          <t>OP-485</t>
+        </is>
+      </c>
+      <c r="I596" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J596" s="2" t="n">
+        <v>46078.71296415881</v>
+      </c>
+      <c r="K596" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>f88a5af1-38ea-44d4-be96-8e36ec8597c9</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>4524f329-85e0-4838-99ef-063f2d97aec9</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E597" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F597" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G597" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H597" t="inlineStr">
+        <is>
+          <t>OP-442</t>
+        </is>
+      </c>
+      <c r="I597" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J597" s="2" t="n">
+        <v>46077.67129749537</v>
+      </c>
+      <c r="K597" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>90cc32d4-6068-4ac3-a118-120c37a4c8b7</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>7e358781-1a40-4444-a375-286af92691c0</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E598" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F598" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G598" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H598" t="inlineStr">
+        <is>
+          <t>OP-401</t>
+        </is>
+      </c>
+      <c r="I598" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J598" s="2" t="n">
+        <v>46087.75463083173</v>
+      </c>
+      <c r="K598" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>ef359209-83db-4ba2-a1f0-dee7e7186a34</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>0e3b467c-d658-4c4d-ab9b-f395d55ef1f8</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E599" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F599" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="G599" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H599" t="inlineStr">
+        <is>
+          <t>OP-216</t>
+        </is>
+      </c>
+      <c r="I599" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J599" s="2" t="n">
+        <v>46064.75463083493</v>
+      </c>
+      <c r="K599" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>06de7f58-9a97-4058-9636-0b0d3b67270b</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>d328b2dc-a7de-4b46-83f1-1808496a8d0c</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E600" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="F600" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G600" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H600" t="inlineStr">
+        <is>
+          <t>OP-669</t>
+        </is>
+      </c>
+      <c r="I600" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J600" s="2" t="n">
+        <v>46065.71296417165</v>
+      </c>
+      <c r="K600" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>88b39549-474c-4365-9209-894b792aa0a2</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>a2b32d8e-f6fb-4f74-bd5d-9ea01cf17cdb</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E601" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F601" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G601" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H601" t="inlineStr">
+        <is>
+          <t>OP-238</t>
+        </is>
+      </c>
+      <c r="I601" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J601" s="2" t="n">
+        <v>46079.83796417471</v>
+      </c>
+      <c r="K601" t="inlineStr">
+        <is>
+          <t>good</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily synthetic data + agent outputs
</commit_message>
<xml_diff>
--- a/decision_log.xlsx
+++ b/decision_log.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1651"/>
+  <dimension ref="A1:K1701"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -82132,7 +82132,7 @@
         </is>
       </c>
       <c r="J1602" s="2" t="n">
-        <v>46061.570378092</v>
+        <v>46061.57037809028</v>
       </c>
       <c r="K1602" t="inlineStr">
         <is>
@@ -82183,7 +82183,7 @@
         </is>
       </c>
       <c r="J1603" s="2" t="n">
-        <v>46088.86204476283</v>
+        <v>46088.86204476852</v>
       </c>
       <c r="K1603" t="inlineStr">
         <is>
@@ -82234,7 +82234,7 @@
         </is>
       </c>
       <c r="J1604" s="2" t="n">
-        <v>46081.73704476601</v>
+        <v>46081.73704476852</v>
       </c>
       <c r="K1604" t="inlineStr">
         <is>
@@ -82285,7 +82285,7 @@
         </is>
       </c>
       <c r="J1605" s="2" t="n">
-        <v>46082.65371143596</v>
+        <v>46082.65371143519</v>
       </c>
       <c r="K1605" t="inlineStr">
         <is>
@@ -82336,7 +82336,7 @@
         </is>
       </c>
       <c r="J1606" s="2" t="n">
-        <v>46068.94537810552</v>
+        <v>46068.94537810185</v>
       </c>
       <c r="K1606" t="inlineStr">
         <is>
@@ -82387,7 +82387,7 @@
         </is>
       </c>
       <c r="J1607" s="2" t="n">
-        <v>46073.69537810851</v>
+        <v>46073.69537811343</v>
       </c>
       <c r="K1607" t="inlineStr">
         <is>
@@ -82438,7 +82438,7 @@
         </is>
       </c>
       <c r="J1608" s="2" t="n">
-        <v>46086.69537811175</v>
+        <v>46086.69537811343</v>
       </c>
       <c r="K1608" t="inlineStr">
         <is>
@@ -82489,7 +82489,7 @@
         </is>
       </c>
       <c r="J1609" s="2" t="n">
-        <v>46084.77871144808</v>
+        <v>46084.77871144676</v>
       </c>
       <c r="K1609" t="inlineStr">
         <is>
@@ -82540,7 +82540,7 @@
         </is>
       </c>
       <c r="J1610" s="2" t="n">
-        <v>46079.77871145105</v>
+        <v>46079.77871144676</v>
       </c>
       <c r="K1610" t="inlineStr">
         <is>
@@ -82591,7 +82591,7 @@
         </is>
       </c>
       <c r="J1611" s="2" t="n">
-        <v>46081.73704478729</v>
+        <v>46081.73704479167</v>
       </c>
       <c r="K1611" t="inlineStr">
         <is>
@@ -82642,7 +82642,7 @@
         </is>
       </c>
       <c r="J1612" s="2" t="n">
-        <v>46083.73704479045</v>
+        <v>46083.73704479167</v>
       </c>
       <c r="K1612" t="inlineStr">
         <is>
@@ -82693,7 +82693,7 @@
         </is>
       </c>
       <c r="J1613" s="2" t="n">
-        <v>46081.61204479326</v>
+        <v>46081.61204479167</v>
       </c>
       <c r="K1613" t="inlineStr">
         <is>
@@ -82744,7 +82744,7 @@
         </is>
       </c>
       <c r="J1614" s="2" t="n">
-        <v>46068.69537812958</v>
+        <v>46068.695378125</v>
       </c>
       <c r="K1614" t="inlineStr">
         <is>
@@ -82795,7 +82795,7 @@
         </is>
       </c>
       <c r="J1615" s="2" t="n">
-        <v>46082.73704479905</v>
+        <v>46082.73704480324</v>
       </c>
       <c r="K1615" t="inlineStr">
         <is>
@@ -82846,7 +82846,7 @@
         </is>
       </c>
       <c r="J1616" s="2" t="n">
-        <v>46072.6537114687</v>
+        <v>46072.65371146991</v>
       </c>
       <c r="K1616" t="inlineStr">
         <is>
@@ -82897,7 +82897,7 @@
         </is>
       </c>
       <c r="J1617" s="2" t="n">
-        <v>46068.8620448049</v>
+        <v>46068.86204480324</v>
       </c>
       <c r="K1617" t="inlineStr">
         <is>
@@ -82948,7 +82948,7 @@
         </is>
       </c>
       <c r="J1618" s="2" t="n">
-        <v>46073.73704480778</v>
+        <v>46073.73704480324</v>
       </c>
       <c r="K1618" t="inlineStr">
         <is>
@@ -82999,7 +82999,7 @@
         </is>
       </c>
       <c r="J1619" s="2" t="n">
-        <v>46064.73704481064</v>
+        <v>46064.73704481481</v>
       </c>
       <c r="K1619" t="inlineStr">
         <is>
@@ -83050,7 +83050,7 @@
         </is>
       </c>
       <c r="J1620" s="2" t="n">
-        <v>46075.77871148023</v>
+        <v>46075.77871148148</v>
       </c>
       <c r="K1620" t="inlineStr">
         <is>
@@ -83101,7 +83101,7 @@
         </is>
       </c>
       <c r="J1621" s="2" t="n">
-        <v>46065.82037814968</v>
+        <v>46065.82037814815</v>
       </c>
       <c r="K1621" t="inlineStr">
         <is>
@@ -83152,7 +83152,7 @@
         </is>
       </c>
       <c r="J1622" s="2" t="n">
-        <v>46063.57037815246</v>
+        <v>46063.57037814815</v>
       </c>
       <c r="K1622" t="inlineStr">
         <is>
@@ -83203,7 +83203,7 @@
         </is>
       </c>
       <c r="J1623" s="2" t="n">
-        <v>46087.57037815528</v>
+        <v>46087.57037815973</v>
       </c>
       <c r="K1623" t="inlineStr">
         <is>
@@ -83254,7 +83254,7 @@
         </is>
       </c>
       <c r="J1624" s="2" t="n">
-        <v>46066.65371149177</v>
+        <v>46066.65371149305</v>
       </c>
       <c r="K1624" t="inlineStr">
         <is>
@@ -83305,7 +83305,7 @@
         </is>
       </c>
       <c r="J1625" s="2" t="n">
-        <v>46065.69537816125</v>
+        <v>46065.69537815973</v>
       </c>
       <c r="K1625" t="inlineStr">
         <is>
@@ -83356,7 +83356,7 @@
         </is>
       </c>
       <c r="J1626" s="2" t="n">
-        <v>46066.7787114974</v>
+        <v>46066.77871149305</v>
       </c>
       <c r="K1626" t="inlineStr">
         <is>
@@ -83407,7 +83407,7 @@
         </is>
       </c>
       <c r="J1627" s="2" t="n">
-        <v>46086.82037816704</v>
+        <v>46086.82037817129</v>
       </c>
       <c r="K1627" t="inlineStr">
         <is>
@@ -83458,7 +83458,7 @@
         </is>
       </c>
       <c r="J1628" s="2" t="n">
-        <v>46074.94537817016</v>
+        <v>46074.94537817129</v>
       </c>
       <c r="K1628" t="inlineStr">
         <is>
@@ -83509,7 +83509,7 @@
         </is>
       </c>
       <c r="J1629" s="2" t="n">
-        <v>46087.77871150631</v>
+        <v>46087.77871150463</v>
       </c>
       <c r="K1629" t="inlineStr">
         <is>
@@ -83560,7 +83560,7 @@
         </is>
       </c>
       <c r="J1630" s="2" t="n">
-        <v>46077.57037817586</v>
+        <v>46077.57037817129</v>
       </c>
       <c r="K1630" t="inlineStr">
         <is>
@@ -83611,7 +83611,7 @@
         </is>
       </c>
       <c r="J1631" s="2" t="n">
-        <v>46073.86204484557</v>
+        <v>46073.86204484953</v>
       </c>
       <c r="K1631" t="inlineStr">
         <is>
@@ -83662,7 +83662,7 @@
         </is>
       </c>
       <c r="J1632" s="2" t="n">
-        <v>46073.73704484868</v>
+        <v>46073.73704484953</v>
       </c>
       <c r="K1632" t="inlineStr">
         <is>
@@ -83713,7 +83713,7 @@
         </is>
       </c>
       <c r="J1633" s="2" t="n">
-        <v>46088.69537818477</v>
+        <v>46088.69537818287</v>
       </c>
       <c r="K1633" t="inlineStr">
         <is>
@@ -83764,7 +83764,7 @@
         </is>
       </c>
       <c r="J1634" s="2" t="n">
-        <v>46073.73704485437</v>
+        <v>46073.73704484953</v>
       </c>
       <c r="K1634" t="inlineStr">
         <is>
@@ -83815,7 +83815,7 @@
         </is>
       </c>
       <c r="J1635" s="2" t="n">
-        <v>46069.77871152383</v>
+        <v>46069.77871152778</v>
       </c>
       <c r="K1635" t="inlineStr">
         <is>
@@ -83866,7 +83866,7 @@
         </is>
       </c>
       <c r="J1636" s="2" t="n">
-        <v>46080.82037819338</v>
+        <v>46080.82037819445</v>
       </c>
       <c r="K1636" t="inlineStr">
         <is>
@@ -83917,7 +83917,7 @@
         </is>
       </c>
       <c r="J1637" s="2" t="n">
-        <v>46061.90371152961</v>
+        <v>46061.90371152778</v>
       </c>
       <c r="K1637" t="inlineStr">
         <is>
@@ -83968,7 +83968,7 @@
         </is>
       </c>
       <c r="J1638" s="2" t="n">
-        <v>46064.69537819903</v>
+        <v>46064.69537819445</v>
       </c>
       <c r="K1638" t="inlineStr">
         <is>
@@ -84019,7 +84019,7 @@
         </is>
       </c>
       <c r="J1639" s="2" t="n">
-        <v>46084.94537820183</v>
+        <v>46084.94537820602</v>
       </c>
       <c r="K1639" t="inlineStr">
         <is>
@@ -84070,7 +84070,7 @@
         </is>
       </c>
       <c r="J1640" s="2" t="n">
-        <v>46067.77871153837</v>
+        <v>46067.77871153935</v>
       </c>
       <c r="K1640" t="inlineStr">
         <is>
@@ -84121,7 +84121,7 @@
         </is>
       </c>
       <c r="J1641" s="2" t="n">
-        <v>46073.82037820783</v>
+        <v>46073.82037820602</v>
       </c>
       <c r="K1641" t="inlineStr">
         <is>
@@ -84172,7 +84172,7 @@
         </is>
       </c>
       <c r="J1642" s="2" t="n">
-        <v>46068.86204487725</v>
+        <v>46068.86204487269</v>
       </c>
       <c r="K1642" t="inlineStr">
         <is>
@@ -84223,7 +84223,7 @@
         </is>
       </c>
       <c r="J1643" s="2" t="n">
-        <v>46065.77871154668</v>
+        <v>46065.77871155093</v>
       </c>
       <c r="K1643" t="inlineStr">
         <is>
@@ -84274,7 +84274,7 @@
         </is>
       </c>
       <c r="J1644" s="2" t="n">
-        <v>46081.69537821649</v>
+        <v>46081.69537821759</v>
       </c>
       <c r="K1644" t="inlineStr">
         <is>
@@ -84325,7 +84325,7 @@
         </is>
       </c>
       <c r="J1645" s="2" t="n">
-        <v>46071.9453782194</v>
+        <v>46071.94537821759</v>
       </c>
       <c r="K1645" t="inlineStr">
         <is>
@@ -84376,7 +84376,7 @@
         </is>
       </c>
       <c r="J1646" s="2" t="n">
-        <v>46069.82037822221</v>
+        <v>46069.82037821759</v>
       </c>
       <c r="K1646" t="inlineStr">
         <is>
@@ -84427,7 +84427,7 @@
         </is>
       </c>
       <c r="J1647" s="2" t="n">
-        <v>46065.94537822509</v>
+        <v>46065.94537822917</v>
       </c>
       <c r="K1647" t="inlineStr">
         <is>
@@ -84478,7 +84478,7 @@
         </is>
       </c>
       <c r="J1648" s="2" t="n">
-        <v>46086.61204489461</v>
+        <v>46086.61204489583</v>
       </c>
       <c r="K1648" t="inlineStr">
         <is>
@@ -84529,7 +84529,7 @@
         </is>
       </c>
       <c r="J1649" s="2" t="n">
-        <v>46075.82037823083</v>
+        <v>46075.82037822917</v>
       </c>
       <c r="K1649" t="inlineStr">
         <is>
@@ -84580,7 +84580,7 @@
         </is>
       </c>
       <c r="J1650" s="2" t="n">
-        <v>46083.90371156701</v>
+        <v>46083.9037115625</v>
       </c>
       <c r="K1650" t="inlineStr">
         <is>
@@ -84631,11 +84631,2561 @@
         </is>
       </c>
       <c r="J1651" s="2" t="n">
-        <v>46061.82037823647</v>
+        <v>46061.82037824074</v>
       </c>
       <c r="K1651" t="inlineStr">
         <is>
           <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>546d2eaa-c51d-4306-ac59-fa948c07ad09</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>57ab6d74-f2aa-4832-9eb1-6ff9d5bf8e3e</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1652" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1652" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F1652" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G1652" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1652" t="inlineStr">
+        <is>
+          <t>OP-498</t>
+        </is>
+      </c>
+      <c r="I1652" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1652" s="2" t="n">
+        <v>46079.0535767574</v>
+      </c>
+      <c r="K1652" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>71c6fadf-ed87-475e-9ea7-0fa7a8186492</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>7923be07-ca5a-46e1-b54f-99074ef66e2c</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1653" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1653" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F1653" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G1653" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1653" t="inlineStr">
+        <is>
+          <t>OP-402</t>
+        </is>
+      </c>
+      <c r="I1653" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1653" s="2" t="n">
+        <v>46074.09524342918</v>
+      </c>
+      <c r="K1653" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>96e81b4a-08b9-46c0-a613-7fb046f2147e</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>4d898aa9-1c65-4b1e-a54b-38b41cea9839</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1654" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1654" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F1654" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G1654" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1654" t="inlineStr">
+        <is>
+          <t>OP-973</t>
+        </is>
+      </c>
+      <c r="I1654" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1654" s="2" t="n">
+        <v>46082.01191009995</v>
+      </c>
+      <c r="K1654" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>fe7cb56f-d15a-4c2a-9f63-0a4801eb239c</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>06e330e3-42c6-473e-8b0c-5609d9c4fd34</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1655" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1655" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="F1655" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G1655" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1655" t="inlineStr">
+        <is>
+          <t>OP-563</t>
+        </is>
+      </c>
+      <c r="I1655" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1655" s="2" t="n">
+        <v>46086.88691010346</v>
+      </c>
+      <c r="K1655" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>ab4facd4-47ff-4f42-a22f-8b8ba1d3e68f</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>5dc314db-1ec4-4fca-a591-3f46528f9e14</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1656" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1656" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F1656" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="G1656" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1656" t="inlineStr">
+        <is>
+          <t>OP-716</t>
+        </is>
+      </c>
+      <c r="I1656" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1656" s="2" t="n">
+        <v>46071.01191010661</v>
+      </c>
+      <c r="K1656" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>2c8483d4-9b1a-45b2-afc6-de2aa53c3606</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>12e7c0d0-038c-4ca1-9dd4-1a58f374423f</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1657" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1657" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F1657" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="G1657" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1657" t="inlineStr">
+        <is>
+          <t>OP-232</t>
+        </is>
+      </c>
+      <c r="I1657" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1657" s="2" t="n">
+        <v>46082.84524344344</v>
+      </c>
+      <c r="K1657" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>4994c1e9-fb2f-4c48-8394-edeeff8cc0be</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>3320910b-fe0c-40dc-a6fa-b2621760955a</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1658" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1658" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F1658" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="G1658" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1658" t="inlineStr">
+        <is>
+          <t>OP-866</t>
+        </is>
+      </c>
+      <c r="I1658" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1658" s="2" t="n">
+        <v>46077.80357677994</v>
+      </c>
+      <c r="K1658" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>2c967c5b-fa23-42e9-8cbb-27f3f80ce7ee</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>b85720b9-16f7-4d68-9800-f5099246c862</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1659" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1659" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="F1659" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G1659" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1659" t="inlineStr">
+        <is>
+          <t>OP-401</t>
+        </is>
+      </c>
+      <c r="I1659" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1659" s="2" t="n">
+        <v>46088.09524344984</v>
+      </c>
+      <c r="K1659" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>b448308d-75c0-4389-a0e9-6e5fb320bc68</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>2562bd8c-c4ae-4098-af74-634b0c20a9bb</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1660" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1660" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="F1660" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G1660" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1660" t="inlineStr">
+        <is>
+          <t>OP-292</t>
+        </is>
+      </c>
+      <c r="I1660" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1660" s="2" t="n">
+        <v>46068.01191012007</v>
+      </c>
+      <c r="K1660" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>61b47140-5ad7-475c-a621-19e3a7b0161a</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>b2043ac9-51b6-4436-9009-2b9441ec57c6</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1661" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1661" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F1661" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G1661" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1661" t="inlineStr">
+        <is>
+          <t>OP-522</t>
+        </is>
+      </c>
+      <c r="I1661" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1661" s="2" t="n">
+        <v>46060.88691012332</v>
+      </c>
+      <c r="K1661" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>6bfe7e68-0fc6-47a9-9367-b1d351c897e0</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>b76145ac-2cca-45d8-8027-848e5228b265</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1662" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1662" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="F1662" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G1662" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1662" t="inlineStr">
+        <is>
+          <t>OP-295</t>
+        </is>
+      </c>
+      <c r="I1662" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1662" s="2" t="n">
+        <v>46083.01191012653</v>
+      </c>
+      <c r="K1662" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>95d212aa-fb3b-4a35-b88b-df7ea0b7ede6</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>579b495e-6d4e-4dbb-83fa-211bcaafc3ed</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1663" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1663" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="F1663" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G1663" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1663" t="inlineStr">
+        <is>
+          <t>OP-703</t>
+        </is>
+      </c>
+      <c r="I1663" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1663" s="2" t="n">
+        <v>46060.84524346314</v>
+      </c>
+      <c r="K1663" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>68b492ec-9727-44ca-a5a6-944209ab7be6</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>12f1af42-93ef-485d-9778-a762bc02b4ae</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1664" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1664" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="F1664" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G1664" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1664" t="inlineStr">
+        <is>
+          <t>OP-184</t>
+        </is>
+      </c>
+      <c r="I1664" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1664" s="2" t="n">
+        <v>46079.09524346657</v>
+      </c>
+      <c r="K1664" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>c32167f7-75f7-4546-8249-a22c328e28dd</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>9b060e97-5aeb-4ba9-9b1a-a0e6e69da063</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1665" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1665" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F1665" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G1665" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1665" t="inlineStr">
+        <is>
+          <t>OP-703</t>
+        </is>
+      </c>
+      <c r="I1665" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1665" s="2" t="n">
+        <v>46071.80357680303</v>
+      </c>
+      <c r="K1665" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>d6531bbf-77ab-4983-9655-5969c971ca62</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>dfe14294-5675-4662-af29-698700b69859</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1666" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1666" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F1666" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G1666" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1666" t="inlineStr">
+        <is>
+          <t>OP-764</t>
+        </is>
+      </c>
+      <c r="I1666" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1666" s="2" t="n">
+        <v>46074.97024347279</v>
+      </c>
+      <c r="K1666" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>b2c52543-a012-4fb8-9002-f1fe8c526686</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>69e7348b-c265-405c-b2f6-2dc28a3eec80</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1667" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1667" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F1667" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G1667" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1667" t="inlineStr">
+        <is>
+          <t>OP-119</t>
+        </is>
+      </c>
+      <c r="I1667" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1667" s="2" t="n">
+        <v>46082.09524347637</v>
+      </c>
+      <c r="K1667" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>f4d2798c-52aa-4c42-8bb4-21c3cc706152</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>21084d39-cd0e-4b0a-8312-fe2471e2ad13</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1668" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1668" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="F1668" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G1668" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1668" t="inlineStr">
+        <is>
+          <t>OP-647</t>
+        </is>
+      </c>
+      <c r="I1668" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1668" s="2" t="n">
+        <v>46070.92857681295</v>
+      </c>
+      <c r="K1668" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>baa572d9-a7c2-4fed-8406-c34685213cdd</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>58878448-5c52-42eb-a195-866fa8bf7e52</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1669" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1669" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F1669" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G1669" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1669" t="inlineStr">
+        <is>
+          <t>OP-839</t>
+        </is>
+      </c>
+      <c r="I1669" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1669" s="2" t="n">
+        <v>46062.80357681617</v>
+      </c>
+      <c r="K1669" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>c042ec70-b38f-4241-88dc-2dc706724c37</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>5c60f1ac-e406-4d09-8556-1b3ee905ebf8</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1670" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1670" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="F1670" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G1670" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1670" t="inlineStr">
+        <is>
+          <t>OP-955</t>
+        </is>
+      </c>
+      <c r="I1670" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1670" s="2" t="n">
+        <v>46071.01191015267</v>
+      </c>
+      <c r="K1670" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>73353992-9c86-475e-b241-723d2ec43935</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>ef6a45c5-4825-49f2-876f-92cb78724d7c</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1671" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1671" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="F1671" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="G1671" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1671" t="inlineStr">
+        <is>
+          <t>OP-162</t>
+        </is>
+      </c>
+      <c r="I1671" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1671" s="2" t="n">
+        <v>46081.80357682281</v>
+      </c>
+      <c r="K1671" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>1f0f6fe8-8f4c-4e1f-87b2-1c9aec54b27e</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>3ead2d53-4ccb-429b-a2a5-e7a68cee8e8a</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1672" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1672" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F1672" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G1672" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1672" t="inlineStr">
+        <is>
+          <t>OP-814</t>
+        </is>
+      </c>
+      <c r="I1672" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1672" s="2" t="n">
+        <v>46070.88691015931</v>
+      </c>
+      <c r="K1672" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>086d75fe-fa8a-4be4-855a-53728f30d4ef</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>0c5f752e-b73b-4645-bf37-c3bbfd9cb7d8</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1673" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1673" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F1673" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G1673" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1673" t="inlineStr">
+        <is>
+          <t>OP-582</t>
+        </is>
+      </c>
+      <c r="I1673" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1673" s="2" t="n">
+        <v>46065.88691016247</v>
+      </c>
+      <c r="K1673" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>3e63e9d2-cc0b-4dbf-9668-fdb653485ce1</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>2449b7e5-78fc-40d4-b51c-7a641035fd87</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1674" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1674" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1674" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G1674" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1674" t="inlineStr">
+        <is>
+          <t>OP-626</t>
+        </is>
+      </c>
+      <c r="I1674" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1674" s="2" t="n">
+        <v>46089.01191016587</v>
+      </c>
+      <c r="K1674" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>be5952c2-844b-4fbd-b499-3634ac508ec9</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>8fd0e957-b0e0-48c7-b5cb-937a005f8741</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1675" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1675" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F1675" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G1675" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1675" t="inlineStr">
+        <is>
+          <t>OP-141</t>
+        </is>
+      </c>
+      <c r="I1675" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1675" s="2" t="n">
+        <v>46071.97024350247</v>
+      </c>
+      <c r="K1675" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>b098279e-d550-4451-9b9e-2f860d18fb08</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>c08bef1a-097c-4d6d-97ce-ace3a2036c13</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1676" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1676" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="F1676" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="G1676" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1676" t="inlineStr">
+        <is>
+          <t>OP-111</t>
+        </is>
+      </c>
+      <c r="I1676" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1676" s="2" t="n">
+        <v>46060.80357683908</v>
+      </c>
+      <c r="K1676" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>6d3817b2-8790-4d42-a4eb-f32278452925</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>70dfe2fc-eeb1-43d9-929d-de1432f0debe</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1677" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1677" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F1677" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G1677" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1677" t="inlineStr">
+        <is>
+          <t>OP-426</t>
+        </is>
+      </c>
+      <c r="I1677" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1677" s="2" t="n">
+        <v>46061.7619101755</v>
+      </c>
+      <c r="K1677" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>83b80d39-2756-44b6-a26e-09fd0ed5800a</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>d8df92f9-4a92-476f-b577-7ed831caf15b</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1678" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1678" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="F1678" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="G1678" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1678" t="inlineStr">
+        <is>
+          <t>OP-274</t>
+        </is>
+      </c>
+      <c r="I1678" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1678" s="2" t="n">
+        <v>46077.8869101791</v>
+      </c>
+      <c r="K1678" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>b0c419c5-05d3-4ee3-a3eb-31a0f43454cb</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>5e4c6806-f63b-48b6-bcb1-715e65bc82fe</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1679" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1679" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="F1679" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G1679" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1679" t="inlineStr">
+        <is>
+          <t>OP-264</t>
+        </is>
+      </c>
+      <c r="I1679" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1679" s="2" t="n">
+        <v>46072.97024351553</v>
+      </c>
+      <c r="K1679" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>de7c8353-3e35-4fc3-86cc-c62fa22c86b4</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>6b6a2616-8905-478f-a523-6cc7cc7e9975</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1680" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1680" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F1680" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G1680" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1680" t="inlineStr">
+        <is>
+          <t>OP-349</t>
+        </is>
+      </c>
+      <c r="I1680" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1680" s="2" t="n">
+        <v>46080.05357685211</v>
+      </c>
+      <c r="K1680" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>d9f9c1e9-bcf8-4b6f-89c4-ab6ce39ebec7</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>92459525-16a6-4d67-805f-6fdf96fcf29d</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1681" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1681" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="F1681" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="G1681" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1681" t="inlineStr">
+        <is>
+          <t>OP-663</t>
+        </is>
+      </c>
+      <c r="I1681" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1681" s="2" t="n">
+        <v>46070.97024352251</v>
+      </c>
+      <c r="K1681" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>64659285-6500-4119-8a18-c70221189591</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>b063787e-7684-48c6-9c66-b68552a50c2a</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1682" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1682" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F1682" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="G1682" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1682" t="inlineStr">
+        <is>
+          <t>OP-103</t>
+        </is>
+      </c>
+      <c r="I1682" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1682" s="2" t="n">
+        <v>46077.05357685918</v>
+      </c>
+      <c r="K1682" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>cc077357-59de-463f-bf23-d707ea748e50</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>ef2bb356-22ba-4a69-b6bd-474dbcd2bfda</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1683" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1683" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F1683" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="G1683" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1683" t="inlineStr">
+        <is>
+          <t>OP-308</t>
+        </is>
+      </c>
+      <c r="I1683" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1683" s="2" t="n">
+        <v>46079.8869101956</v>
+      </c>
+      <c r="K1683" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>40696172-742f-465b-b34b-5be777fbe725</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>c7dd6d71-5a7a-4f0d-a69b-881815587ddf</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1684" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1684" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F1684" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G1684" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1684" t="inlineStr">
+        <is>
+          <t>OP-647</t>
+        </is>
+      </c>
+      <c r="I1684" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1684" s="2" t="n">
+        <v>46083.01191019875</v>
+      </c>
+      <c r="K1684" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>c59082a4-040c-4397-bf31-49df5c01f9f5</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>1b9426e0-dc1d-49ec-bb71-5dc56c29d85d</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1685" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1685" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F1685" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G1685" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1685" t="inlineStr">
+        <is>
+          <t>OP-743</t>
+        </is>
+      </c>
+      <c r="I1685" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1685" s="2" t="n">
+        <v>46077.05357686911</v>
+      </c>
+      <c r="K1685" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>0a797b11-232d-4cbf-9a78-2f58ef5e08c9</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>260bc29a-d52a-43f3-ab31-c7a7ef019d16</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1686" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1686" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F1686" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G1686" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1686" t="inlineStr">
+        <is>
+          <t>OP-321</t>
+        </is>
+      </c>
+      <c r="I1686" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1686" s="2" t="n">
+        <v>46087.88691020555</v>
+      </c>
+      <c r="K1686" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>8a8d0f88-92a3-4e63-8659-3a924eae8001</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>06bab144-a675-4a7d-bd87-79014aedc371</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1687" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1687" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F1687" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="G1687" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1687" t="inlineStr">
+        <is>
+          <t>OP-461</t>
+        </is>
+      </c>
+      <c r="I1687" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1687" s="2" t="n">
+        <v>46078.97024354199</v>
+      </c>
+      <c r="K1687" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>b1bd0d3c-0df0-4ff9-9b22-7d3cf086d115</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>4a697c78-2548-4eec-be93-c019ec24998b</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1688" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1688" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="F1688" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G1688" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1688" t="inlineStr">
+        <is>
+          <t>OP-219</t>
+        </is>
+      </c>
+      <c r="I1688" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1688" s="2" t="n">
+        <v>46069.88691021168</v>
+      </c>
+      <c r="K1688" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>77a11c19-c711-4cd3-b223-7991e748397c</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>794b3f5d-2b87-45f8-9f5d-540c3ccbb0c9</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1689" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1689" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="F1689" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G1689" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1689" t="inlineStr">
+        <is>
+          <t>OP-436</t>
+        </is>
+      </c>
+      <c r="I1689" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1689" s="2" t="n">
+        <v>46077.01191021502</v>
+      </c>
+      <c r="K1689" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>6a90a976-6c33-4007-a6be-7858a3b1c4b8</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>dd2423ec-5c50-4b40-8941-591a214a1726</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1690" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1690" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="F1690" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G1690" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1690" t="inlineStr">
+        <is>
+          <t>OP-247</t>
+        </is>
+      </c>
+      <c r="I1690" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1690" s="2" t="n">
+        <v>46079.92857688489</v>
+      </c>
+      <c r="K1690" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>32b5bcb6-44e6-464f-9e77-ddfe056a97fc</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>99b9ea5f-acab-42d1-a108-88ca690492f9</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1691" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1691" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="F1691" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G1691" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1691" t="inlineStr">
+        <is>
+          <t>OP-451</t>
+        </is>
+      </c>
+      <c r="I1691" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1691" s="2" t="n">
+        <v>46080.80357688816</v>
+      </c>
+      <c r="K1691" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>c4c45376-a6c7-48d0-9668-c1638422e454</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>4a4bd5ff-b415-4f34-ac73-d84b8e657757</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1692" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1692" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F1692" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="G1692" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1692" t="inlineStr">
+        <is>
+          <t>OP-825</t>
+        </is>
+      </c>
+      <c r="I1692" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1692" s="2" t="n">
+        <v>46088.88691022486</v>
+      </c>
+      <c r="K1692" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>46f17afc-4e0e-4134-9dbb-7f9f642978b2</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>0f9bc35e-a2cd-4f1d-8d76-3e1d23bf416b</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1693" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1693" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F1693" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G1693" t="inlineStr">
+        <is>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="H1693" t="inlineStr">
+        <is>
+          <t>OP-651</t>
+        </is>
+      </c>
+      <c r="I1693" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1693" s="2" t="n">
+        <v>46071.05357689474</v>
+      </c>
+      <c r="K1693" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>20e49761-167a-472e-a477-cd5f0dc851f4</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>1d279b40-4d75-4083-8567-f2de1634e430</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1694" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1694" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="F1694" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G1694" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1694" t="inlineStr">
+        <is>
+          <t>OP-653</t>
+        </is>
+      </c>
+      <c r="I1694" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1694" s="2" t="n">
+        <v>46087.76191023138</v>
+      </c>
+      <c r="K1694" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>e5ad0a14-bf24-4ecc-9bc4-cf3efa91f408</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>2fb1608f-059c-42f9-8705-575d4c58a877</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1695" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1695" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="F1695" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="G1695" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1695" t="inlineStr">
+        <is>
+          <t>OP-358</t>
+        </is>
+      </c>
+      <c r="I1695" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1695" s="2" t="n">
+        <v>46075.92857690123</v>
+      </c>
+      <c r="K1695" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>e179c128-270c-4844-bf39-bf6b21ff53bd</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>c1eef5b2-75f6-43b0-b8e6-461d99ac512b</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1696" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1696" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="F1696" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G1696" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1696" t="inlineStr">
+        <is>
+          <t>OP-694</t>
+        </is>
+      </c>
+      <c r="I1696" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1696" s="2" t="n">
+        <v>46065.72024357169</v>
+      </c>
+      <c r="K1696" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>829680ec-83e1-4fcf-a391-3c4f4c2f741e</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>949ebc06-2a8a-4987-a932-6fd616a8aa81</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1697" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1697" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F1697" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G1697" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1697" t="inlineStr">
+        <is>
+          <t>OP-668</t>
+        </is>
+      </c>
+      <c r="I1697" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1697" s="2" t="n">
+        <v>46067.72024357478</v>
+      </c>
+      <c r="K1697" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>fecee184-b926-4a60-a1a9-d9b08e7c0075</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>6a1a7d08-fada-4ce2-a11f-5245489f4c6f</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>ComplianceAgent</t>
+        </is>
+      </c>
+      <c r="D1698" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1698" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="F1698" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="G1698" t="inlineStr">
+        <is>
+          <t>approved</t>
+        </is>
+      </c>
+      <c r="H1698" t="inlineStr">
+        <is>
+          <t>OP-260</t>
+        </is>
+      </c>
+      <c r="I1698" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1698" s="2" t="n">
+        <v>46083.72024357798</v>
+      </c>
+      <c r="K1698" t="inlineStr">
+        <is>
+          <t>good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>913229aa-2a78-4e8b-9234-3e48295fac7e</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>944c66d7-f53a-4cd6-9511-159698cd4419</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>MonitoringAgent</t>
+        </is>
+      </c>
+      <c r="D1699" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1699" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="F1699" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="G1699" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1699" t="inlineStr">
+        <is>
+          <t>OP-804</t>
+        </is>
+      </c>
+      <c r="I1699" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1699" s="2" t="n">
+        <v>46088.01191024825</v>
+      </c>
+      <c r="K1699" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>4165c738-6227-4421-8514-88303264844b</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>41a4f48d-0e68-4c42-9660-515a903adaa2</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1700" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1700" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="F1700" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G1700" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1700" t="inlineStr">
+        <is>
+          <t>OP-364</t>
+        </is>
+      </c>
+      <c r="I1700" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1700" s="2" t="n">
+        <v>46084.84524358477</v>
+      </c>
+      <c r="K1700" t="inlineStr">
+        <is>
+          <t>poor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>7ed3a925-cc98-4925-a2de-9d1d807a1203</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>973218a7-b805-4dfb-8a1b-df529cffde50</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>RiskAgent</t>
+        </is>
+      </c>
+      <c r="D1701" t="inlineStr">
+        <is>
+          <t>Increase cooling / reroute shipment</t>
+        </is>
+      </c>
+      <c r="E1701" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="F1701" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G1701" t="inlineStr">
+        <is>
+          <t>modified</t>
+        </is>
+      </c>
+      <c r="H1701" t="inlineStr">
+        <is>
+          <t>OP-811</t>
+        </is>
+      </c>
+      <c r="I1701" t="inlineStr">
+        <is>
+          <t>Synthetic operator note</t>
+        </is>
+      </c>
+      <c r="J1701" s="2" t="n">
+        <v>46081.01191025465</v>
+      </c>
+      <c r="K1701" t="inlineStr">
+        <is>
+          <t>good</t>
         </is>
       </c>
     </row>

</xml_diff>